<commit_message>
ISSUE-CELLSCLOUD-14149: Development, test Aspose.Cells Cloud SDK for .Net with AI.
</commit_message>
<xml_diff>
--- a/TestData/Book1.xlsx
+++ b/TestData/Book1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\aspose\cells\cloud\src\testdata\Cells\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cells.cloud.family\cells.cloud\src\testdata\Cells\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CAC6793-BD49-46ED-A252-75A83DDD28AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{506BB17B-6CF2-478D-8511-3D14ED0A0AEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="Sheet6" sheetId="6" r:id="rId6"/>
     <sheet name="Sheet7" sheetId="7" r:id="rId7"/>
     <sheet name="Sheet8" sheetId="8" r:id="rId8"/>
+    <sheet name="Sheet9" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Sheet5!$B$3:$E$18</definedName>
@@ -101,7 +102,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="37">
   <si>
     <t>aspose</t>
   </si>
@@ -210,22 +211,26 @@
   <si>
     <t>Column7</t>
   </si>
+  <si>
+    <t xml:space="preserve">   Hi,     RoY   Wang.  hellow  word!     
+</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_ &quot;¥&quot;* #,##0_ ;_ &quot;¥&quot;* \-#,##0_ ;_ &quot;¥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;¥&quot;* #,##0.00_ ;_ &quot;¥&quot;* \-#,##0.00_ ;_ &quot;¥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="_ &quot;¥&quot;* #,##0_ ;_ &quot;¥&quot;* \-#,##0_ ;_ &quot;¥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="166" formatCode="_ &quot;¥&quot;* #,##0.00_ ;_ &quot;¥&quot;* \-#,##0.00_ ;_ &quot;¥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="167" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -239,7 +244,7 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="宋体"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -263,7 +268,7 @@
     </font>
     <font>
       <sz val="9"/>
-      <name val="宋体"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -295,26 +300,26 @@
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -328,12 +333,6 @@
     <cellStyle name="Percent" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
   <dxfs count="5">
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -363,6 +362,12 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -410,7 +415,7 @@
               </a:solidFill>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="zh-CN"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -532,7 +537,7 @@
           </a:solidFill>
         </a:defRPr>
       </a:pPr>
-      <a:endParaRPr lang="zh-CN"/>
+      <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -582,7 +587,7 @@
               <a:cs typeface="Calibri"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="zh-CN"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -785,7 +790,7 @@
                 <a:cs typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="zh-CN"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="12186015"/>
@@ -842,7 +847,7 @@
                 <a:cs typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="zh-CN"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="7764587"/>
@@ -882,7 +887,7 @@
               <a:cs typeface="Calibri"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="zh-CN"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -951,7 +956,7 @@
               <a:cs typeface="Calibri"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="zh-CN"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -1010,7 +1015,7 @@
                     <a:cs typeface="Calibri"/>
                   </a:defRPr>
                 </a:pPr>
-                <a:endParaRPr lang="zh-CN"/>
+                <a:endParaRPr lang="en-US"/>
               </a:p>
             </c:txPr>
             <c:dLblPos val="t"/>
@@ -1209,7 +1214,7 @@
                 <a:cs typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="zh-CN"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="56946769"/>
@@ -1266,7 +1271,7 @@
                 <a:cs typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="zh-CN"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="63849291"/>
@@ -1293,7 +1298,7 @@
           <a:bodyPr rot="0" vert="horz"/>
           <a:lstStyle/>
           <a:p>
-            <a:pPr>
+            <a:pPr rtl="0">
               <a:defRPr lang="en-US" sz="900" b="0" i="0" u="none" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
@@ -1306,7 +1311,7 @@
                 <a:cs typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="zh-CN"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
       </c:dTable>
@@ -1343,7 +1348,7 @@
               <a:cs typeface="Calibri"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="zh-CN"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -1412,7 +1417,7 @@
               <a:cs typeface="Calibri"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="zh-CN"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -1678,7 +1683,7 @@
                 <a:cs typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="zh-CN"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="34701889"/>
@@ -1735,7 +1740,7 @@
                 <a:cs typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="zh-CN"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="23605975"/>
@@ -1775,7 +1780,7 @@
               <a:cs typeface="Calibri"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="zh-CN"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:legend>
@@ -4990,8 +4995,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="887492" y="500"/>
-          <a:ext cx="1896902" cy="1138141"/>
+          <a:off x="563770" y="1143"/>
+          <a:ext cx="2115721" cy="1269433"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5032,12 +5037,12 @@
         </a:fontRef>
       </dsp:style>
       <dsp:txBody>
-        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="175260" tIns="175260" rIns="175260" bIns="175260" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
+        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="194310" tIns="194310" rIns="194310" bIns="194310" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" defTabSz="2044700">
+          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" defTabSz="2266950">
             <a:lnSpc>
               <a:spcPct val="90000"/>
             </a:lnSpc>
@@ -5050,14 +5055,14 @@
             <a:buNone/>
           </a:pPr>
           <a:r>
-            <a:rPr lang="en-US" sz="4600" kern="1200"/>
+            <a:rPr lang="en-US" sz="5100" kern="1200"/>
             <a:t>Cells</a:t>
           </a:r>
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="887492" y="500"/>
-        <a:ext cx="1896902" cy="1138141"/>
+        <a:off x="563770" y="1143"/>
+        <a:ext cx="2115721" cy="1269433"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{5C25943E-09F9-4D35-8A3B-0E199ABC8277}">
@@ -5067,8 +5072,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="887492" y="1328332"/>
-          <a:ext cx="1896902" cy="1138141"/>
+          <a:off x="563770" y="1482148"/>
+          <a:ext cx="2115721" cy="1269433"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5109,12 +5114,12 @@
         </a:fontRef>
       </dsp:style>
       <dsp:txBody>
-        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="175260" tIns="175260" rIns="175260" bIns="175260" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
+        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="194310" tIns="194310" rIns="194310" bIns="194310" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" defTabSz="2044700">
+          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" defTabSz="2266950">
             <a:lnSpc>
               <a:spcPct val="90000"/>
             </a:lnSpc>
@@ -5127,14 +5132,14 @@
             <a:buNone/>
           </a:pPr>
           <a:r>
-            <a:rPr lang="en-US" sz="4600" kern="1200"/>
+            <a:rPr lang="en-US" sz="5100" kern="1200"/>
             <a:t>Words</a:t>
           </a:r>
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="887492" y="1328332"/>
-        <a:ext cx="1896902" cy="1138141"/>
+        <a:off x="563770" y="1482148"/>
+        <a:ext cx="2115721" cy="1269433"/>
       </dsp:txXfrm>
     </dsp:sp>
   </dsp:spTree>
@@ -5156,8 +5161,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm rot="5400000">
-          <a:off x="2374498" y="60888"/>
-          <a:ext cx="917091" cy="797869"/>
+          <a:off x="2004230" y="67577"/>
+          <a:ext cx="1015751" cy="883704"/>
         </a:xfrm>
         <a:prstGeom prst="hexagon">
           <a:avLst>
@@ -5201,12 +5206,12 @@
         </a:fontRef>
       </dsp:style>
       <dsp:txBody>
-        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="57150" tIns="57150" rIns="57150" bIns="57150" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
+        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="60960" tIns="60960" rIns="60960" bIns="60960" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" defTabSz="666750">
+          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" defTabSz="711200">
             <a:lnSpc>
               <a:spcPct val="90000"/>
             </a:lnSpc>
@@ -5218,12 +5223,12 @@
             </a:spcAft>
             <a:buNone/>
           </a:pPr>
-          <a:endParaRPr lang="en-US" sz="1500" kern="1200"/>
+          <a:endParaRPr lang="en-US" sz="1600" kern="1200"/>
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm rot="-5400000">
-        <a:off x="2558444" y="144190"/>
-        <a:ext cx="549199" cy="631265"/>
+        <a:off x="2207964" y="159842"/>
+        <a:ext cx="608282" cy="699175"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{B930369B-D2A0-4F63-9F48-D9B1B51F9A4E}">
@@ -5233,8 +5238,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="3256190" y="184695"/>
-          <a:ext cx="1023473" cy="550254"/>
+          <a:off x="2980774" y="204704"/>
+          <a:ext cx="1133579" cy="609451"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5258,12 +5263,12 @@
         <a:fontRef idx="minor"/>
       </dsp:style>
       <dsp:txBody>
-        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="95250" tIns="95250" rIns="95250" bIns="95250" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
+        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="106680" tIns="106680" rIns="106680" bIns="106680" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr marL="0" lvl="0" indent="0" algn="l" defTabSz="1111250">
+          <a:pPr marL="0" lvl="0" indent="0" algn="l" defTabSz="1244600">
             <a:lnSpc>
               <a:spcPct val="90000"/>
             </a:lnSpc>
@@ -5275,12 +5280,12 @@
             </a:spcAft>
             <a:buNone/>
           </a:pPr>
-          <a:endParaRPr lang="en-US" sz="2500" kern="1200"/>
+          <a:endParaRPr lang="en-US" sz="2800" kern="1200"/>
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="3256190" y="184695"/>
-        <a:ext cx="1023473" cy="550254"/>
+        <a:off x="2980774" y="204704"/>
+        <a:ext cx="1133579" cy="609451"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{53337A83-2C88-47CB-8EA7-8DEB9E392E35}">
@@ -5290,8 +5295,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm rot="5400000">
-          <a:off x="1512799" y="60888"/>
-          <a:ext cx="917091" cy="797869"/>
+          <a:off x="1049829" y="67577"/>
+          <a:ext cx="1015751" cy="883704"/>
         </a:xfrm>
         <a:prstGeom prst="hexagon">
           <a:avLst>
@@ -5356,8 +5361,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm rot="-5400000">
-        <a:off x="1696745" y="144190"/>
-        <a:ext cx="549199" cy="631265"/>
+        <a:off x="1253563" y="159842"/>
+        <a:ext cx="608282" cy="699175"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{647BCE6B-49D9-4061-808E-497371A775C8}">
@@ -5367,8 +5372,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm rot="5400000">
-          <a:off x="1941998" y="839315"/>
-          <a:ext cx="917091" cy="797869"/>
+          <a:off x="1525201" y="929747"/>
+          <a:ext cx="1015751" cy="883704"/>
         </a:xfrm>
         <a:prstGeom prst="hexagon">
           <a:avLst>
@@ -5412,12 +5417,12 @@
         </a:fontRef>
       </dsp:style>
       <dsp:txBody>
-        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="57150" tIns="57150" rIns="57150" bIns="57150" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
+        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="60960" tIns="60960" rIns="60960" bIns="60960" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" defTabSz="666750">
+          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" defTabSz="711200">
             <a:lnSpc>
               <a:spcPct val="90000"/>
             </a:lnSpc>
@@ -5429,12 +5434,12 @@
             </a:spcAft>
             <a:buNone/>
           </a:pPr>
-          <a:endParaRPr lang="en-US" sz="1500" kern="1200"/>
+          <a:endParaRPr lang="en-US" sz="1600" kern="1200"/>
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm rot="-5400000">
-        <a:off x="2125944" y="922617"/>
-        <a:ext cx="549199" cy="631265"/>
+        <a:off x="1728935" y="1022012"/>
+        <a:ext cx="608282" cy="699175"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{E69DED3E-1798-498A-B9A6-EC95C7494A6D}">
@@ -5444,8 +5449,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="978135" y="963122"/>
-          <a:ext cx="990458" cy="550254"/>
+          <a:off x="457646" y="1066874"/>
+          <a:ext cx="1097012" cy="609451"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5469,12 +5474,12 @@
         <a:fontRef idx="minor"/>
       </dsp:style>
       <dsp:txBody>
-        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="95250" tIns="95250" rIns="95250" bIns="95250" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
+        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="106680" tIns="106680" rIns="106680" bIns="106680" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr marL="0" lvl="0" indent="0" algn="r" defTabSz="1111250">
+          <a:pPr marL="0" lvl="0" indent="0" algn="r" defTabSz="1244600">
             <a:lnSpc>
               <a:spcPct val="90000"/>
             </a:lnSpc>
@@ -5486,12 +5491,12 @@
             </a:spcAft>
             <a:buNone/>
           </a:pPr>
-          <a:endParaRPr lang="en-US" sz="2500" kern="1200"/>
+          <a:endParaRPr lang="en-US" sz="2800" kern="1200"/>
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="978135" y="963122"/>
-        <a:ext cx="990458" cy="550254"/>
+        <a:off x="457646" y="1066874"/>
+        <a:ext cx="1097012" cy="609451"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{8FC7D08A-84F9-4114-9F68-EAA65B3092AA}">
@@ -5501,8 +5506,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm rot="5400000">
-          <a:off x="2803697" y="839315"/>
-          <a:ext cx="917091" cy="797869"/>
+          <a:off x="2479602" y="929747"/>
+          <a:ext cx="1015751" cy="883704"/>
         </a:xfrm>
         <a:prstGeom prst="hexagon">
           <a:avLst>
@@ -5567,8 +5572,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm rot="-5400000">
-        <a:off x="2987643" y="922617"/>
-        <a:ext cx="549199" cy="631265"/>
+        <a:off x="2683336" y="1022012"/>
+        <a:ext cx="608282" cy="699175"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{B7F626B2-5CA0-4456-B060-5D90A1C6F809}">
@@ -5578,8 +5583,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm rot="5400000">
-          <a:off x="2374498" y="1617742"/>
-          <a:ext cx="917091" cy="797869"/>
+          <a:off x="2004230" y="1791918"/>
+          <a:ext cx="1015751" cy="883704"/>
         </a:xfrm>
         <a:prstGeom prst="hexagon">
           <a:avLst>
@@ -5623,12 +5628,12 @@
         </a:fontRef>
       </dsp:style>
       <dsp:txBody>
-        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="57150" tIns="57150" rIns="57150" bIns="57150" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
+        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="60960" tIns="60960" rIns="60960" bIns="60960" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" defTabSz="666750">
+          <a:pPr marL="0" lvl="0" indent="0" algn="ctr" defTabSz="711200">
             <a:lnSpc>
               <a:spcPct val="90000"/>
             </a:lnSpc>
@@ -5640,12 +5645,12 @@
             </a:spcAft>
             <a:buNone/>
           </a:pPr>
-          <a:endParaRPr lang="en-US" sz="1500" kern="1200"/>
+          <a:endParaRPr lang="en-US" sz="1600" kern="1200"/>
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm rot="-5400000">
-        <a:off x="2558444" y="1701044"/>
-        <a:ext cx="549199" cy="631265"/>
+        <a:off x="2207964" y="1884183"/>
+        <a:ext cx="608282" cy="699175"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{F941179A-7E65-4142-A4DE-C77422569540}">
@@ -5655,8 +5660,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="3256190" y="1741549"/>
-          <a:ext cx="1023473" cy="550254"/>
+          <a:off x="2980774" y="1929044"/>
+          <a:ext cx="1133579" cy="609451"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5680,12 +5685,12 @@
         <a:fontRef idx="minor"/>
       </dsp:style>
       <dsp:txBody>
-        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="95250" tIns="95250" rIns="95250" bIns="95250" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
+        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="106680" tIns="106680" rIns="106680" bIns="106680" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr marL="0" lvl="0" indent="0" algn="l" defTabSz="1111250">
+          <a:pPr marL="0" lvl="0" indent="0" algn="l" defTabSz="1244600">
             <a:lnSpc>
               <a:spcPct val="90000"/>
             </a:lnSpc>
@@ -5697,12 +5702,12 @@
             </a:spcAft>
             <a:buNone/>
           </a:pPr>
-          <a:endParaRPr lang="en-US" sz="2500" kern="1200"/>
+          <a:endParaRPr lang="en-US" sz="2800" kern="1200"/>
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="3256190" y="1741549"/>
-        <a:ext cx="1023473" cy="550254"/>
+        <a:off x="2980774" y="1929044"/>
+        <a:ext cx="1133579" cy="609451"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{E548E58E-B118-4D34-9B17-B7C7F1C4A379}">
@@ -5712,8 +5717,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm rot="5400000">
-          <a:off x="1512799" y="1617742"/>
-          <a:ext cx="917091" cy="797869"/>
+          <a:off x="1049829" y="1791918"/>
+          <a:ext cx="1015751" cy="883704"/>
         </a:xfrm>
         <a:prstGeom prst="hexagon">
           <a:avLst>
@@ -5778,8 +5783,8 @@
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm rot="-5400000">
-        <a:off x="1696745" y="1701044"/>
-        <a:ext cx="549199" cy="631265"/>
+        <a:off x="1253563" y="1884183"/>
+        <a:ext cx="608282" cy="699175"/>
       </dsp:txXfrm>
     </dsp:sp>
   </dsp:spTree>
@@ -5801,8 +5806,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="0" y="327810"/>
-          <a:ext cx="5257800" cy="453600"/>
+          <a:off x="0" y="359999"/>
+          <a:ext cx="4572000" cy="504000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5849,8 +5854,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="262890" y="62130"/>
-          <a:ext cx="3680460" cy="531360"/>
+          <a:off x="228600" y="64799"/>
+          <a:ext cx="3200400" cy="590400"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -5891,12 +5896,12 @@
         </a:fontRef>
       </dsp:style>
       <dsp:txBody>
-        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="139113" tIns="0" rIns="139113" bIns="0" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
+        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="120968" tIns="0" rIns="120968" bIns="0" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr marL="0" lvl="0" indent="0" algn="l" defTabSz="800100">
+          <a:pPr marL="0" lvl="0" indent="0" algn="l" defTabSz="889000">
             <a:lnSpc>
               <a:spcPct val="90000"/>
             </a:lnSpc>
@@ -5908,12 +5913,12 @@
             </a:spcAft>
             <a:buNone/>
           </a:pPr>
-          <a:endParaRPr lang="en-US" sz="1800" kern="1200"/>
+          <a:endParaRPr lang="en-US" sz="2000" kern="1200"/>
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="288829" y="88069"/>
-        <a:ext cx="3628582" cy="479482"/>
+        <a:off x="257421" y="93620"/>
+        <a:ext cx="3142758" cy="532758"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{9A40B308-CE02-4B71-BA70-C0D200CBD383}">
@@ -5923,8 +5928,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="0" y="1144290"/>
-          <a:ext cx="5257800" cy="453600"/>
+          <a:off x="0" y="1267200"/>
+          <a:ext cx="4572000" cy="504000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5971,8 +5976,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="262890" y="878610"/>
-          <a:ext cx="3680460" cy="531360"/>
+          <a:off x="228600" y="972000"/>
+          <a:ext cx="3200400" cy="590400"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -6013,12 +6018,12 @@
         </a:fontRef>
       </dsp:style>
       <dsp:txBody>
-        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="139113" tIns="0" rIns="139113" bIns="0" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
+        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="120968" tIns="0" rIns="120968" bIns="0" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr marL="0" lvl="0" indent="0" algn="l" defTabSz="800100">
+          <a:pPr marL="0" lvl="0" indent="0" algn="l" defTabSz="889000">
             <a:lnSpc>
               <a:spcPct val="90000"/>
             </a:lnSpc>
@@ -6030,12 +6035,12 @@
             </a:spcAft>
             <a:buNone/>
           </a:pPr>
-          <a:endParaRPr lang="en-US" sz="1800" kern="1200"/>
+          <a:endParaRPr lang="en-US" sz="2000" kern="1200"/>
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="288829" y="904549"/>
-        <a:ext cx="3628582" cy="479482"/>
+        <a:off x="257421" y="1000821"/>
+        <a:ext cx="3142758" cy="532758"/>
       </dsp:txXfrm>
     </dsp:sp>
     <dsp:sp modelId="{BE4CD07D-369F-49DD-8139-FD09651870C8}">
@@ -6045,8 +6050,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="0" y="1960770"/>
-          <a:ext cx="5257800" cy="453600"/>
+          <a:off x="0" y="2174400"/>
+          <a:ext cx="4572000" cy="504000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6093,8 +6098,8 @@
       </dsp:nvSpPr>
       <dsp:spPr>
         <a:xfrm>
-          <a:off x="262890" y="1695090"/>
-          <a:ext cx="3680460" cy="531360"/>
+          <a:off x="228600" y="1879200"/>
+          <a:ext cx="3200400" cy="590400"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -6135,12 +6140,12 @@
         </a:fontRef>
       </dsp:style>
       <dsp:txBody>
-        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="139113" tIns="0" rIns="139113" bIns="0" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
+        <a:bodyPr spcFirstLastPara="0" vert="horz" wrap="square" lIns="120968" tIns="0" rIns="120968" bIns="0" numCol="1" spcCol="1270" anchor="ctr" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr marL="0" lvl="0" indent="0" algn="l" defTabSz="800100">
+          <a:pPr marL="0" lvl="0" indent="0" algn="l" defTabSz="889000">
             <a:lnSpc>
               <a:spcPct val="90000"/>
             </a:lnSpc>
@@ -6152,12 +6157,12 @@
             </a:spcAft>
             <a:buNone/>
           </a:pPr>
-          <a:endParaRPr lang="en-US" sz="1800" kern="1200"/>
+          <a:endParaRPr lang="en-US" sz="2000" kern="1200"/>
         </a:p>
       </dsp:txBody>
       <dsp:txXfrm>
-        <a:off x="288829" y="1721029"/>
-        <a:ext cx="3628582" cy="479482"/>
+        <a:off x="257421" y="1908021"/>
+        <a:ext cx="3142758" cy="532758"/>
       </dsp:txXfrm>
     </dsp:sp>
   </dsp:spTree>
@@ -10208,16 +10213,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>376237</xdr:colOff>
-      <xdr:row>49</xdr:row>
-      <xdr:rowOff>157162</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>223837</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>100012</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>71437</xdr:colOff>
-      <xdr:row>64</xdr:row>
-      <xdr:rowOff>42862</xdr:rowOff>
+      <xdr:colOff>528637</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>176212</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -11375,7 +11380,7 @@
         <xdr:cNvPr id="4" name="Picture 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6C9FAE5B-687B-188C-0EA2-F6CADF7C07A8}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000004000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -11430,8 +11435,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table1" displayName="Table1" ref="M6:P10" totalsRowShown="0">
   <autoFilter ref="M6:P10" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Column1" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Column2" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Column1" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Column2" dataDxfId="3"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Column3"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Column4"/>
   </tableColumns>
@@ -11440,9 +11445,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -11480,9 +11485,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -11515,26 +11520,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -11567,26 +11555,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -11761,7 +11732,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:T39"/>
-  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <sheetData>
     <row r="2" spans="2:20">
       <c r="P2" s="8"/>
@@ -11879,15 +11850,18 @@
       </iconSet>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G15:I19 K20:L21">
-    <cfRule type="cellIs" dxfId="4" priority="4" operator="lessThan">
-      <formula>"w"</formula>
+  <conditionalFormatting sqref="D30:G34 I34:J35 M35 L35:L36 L38 J41 F41">
+    <cfRule type="top10" dxfId="2" priority="1" percent="1" rank="10"/>
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="5" operator="greaterThan">
-      <formula>1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D30:G34 I34:J35 M35 L35:L36 L38 J41 F41">
     <cfRule type="dataBar" priority="7">
       <dataBar>
         <cfvo type="min"/>
@@ -11901,20 +11875,13 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D30:G34 I34:J35 M35 L35:L36 L38 J41 F41">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF5A8AC6"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
+  <conditionalFormatting sqref="G15:I19 K20:L21">
+    <cfRule type="cellIs" dxfId="1" priority="4" operator="lessThan">
+      <formula>"w"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D30:G34 I34:J35 M35 L35:L36 L38 J41 F41">
-    <cfRule type="top10" dxfId="2" priority="1" percent="1" rank="10"/>
+    <cfRule type="cellIs" dxfId="0" priority="5" operator="greaterThan">
+      <formula>1</formula>
+    </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -11965,11 +11932,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B5:H14"/>
-  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="13.5"/>
+  <dimension ref="B5:H15"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="6" max="7" width="15.625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="5" spans="2:8">
@@ -11979,7 +11946,7 @@
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
     </row>
-    <row r="8" spans="2:8" ht="14.25">
+    <row r="8" spans="2:8">
       <c r="G8" t="s">
         <v>3</v>
       </c>
@@ -11990,7 +11957,7 @@
     <row r="10" spans="2:8">
       <c r="F10" s="4">
         <f ca="1">NOW()</f>
-        <v>44706.569663657407</v>
+        <v>45539.845608101852</v>
       </c>
     </row>
     <row r="12" spans="2:8">
@@ -12004,6 +11971,11 @@
     <row r="14" spans="2:8">
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
+    </row>
+    <row r="15" spans="2:8" ht="195">
+      <c r="F15" s="7" t="s">
+        <v>36</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -12019,7 +11991,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="E15:F21"/>
-  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <sheetData>
     <row r="15" spans="5:6">
       <c r="E15" t="s">
@@ -12088,7 +12060,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="C7:D11"/>
-  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <sheetData>
     <row r="7" spans="3:4">
       <c r="C7" t="s">
@@ -12143,9 +12115,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr filterMode="1"/>
   <dimension ref="B3:E18"/>
-  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="10.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:5">
@@ -12395,7 +12367,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="S3:AC14"/>
-  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <sheetData>
     <row r="3" spans="19:29"/>
     <row r="13" spans="19:29">
@@ -12534,10 +12506,10 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="C3:P23"/>
-  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="9" width="10.875" customWidth="1"/>
-    <col min="13" max="16" width="10.875" customWidth="1"/>
+    <col min="3" max="9" width="10.85546875" customWidth="1"/>
+    <col min="13" max="16" width="10.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="3:16">
@@ -12631,10 +12603,10 @@
       <c r="I6">
         <v>3</v>
       </c>
-      <c r="M6" s="7" t="s">
+      <c r="M6" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="N6" s="7" t="s">
+      <c r="N6" s="3" t="s">
         <v>30</v>
       </c>
       <c r="O6" t="s">
@@ -12666,8 +12638,8 @@
       <c r="I7">
         <v>4</v>
       </c>
-      <c r="M7" s="7"/>
-      <c r="N7" s="7"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
     </row>
     <row r="8" spans="3:16">
       <c r="C8">
@@ -12691,8 +12663,8 @@
       <c r="I8">
         <v>5</v>
       </c>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
     </row>
     <row r="9" spans="3:16">
       <c r="C9">
@@ -12716,8 +12688,8 @@
       <c r="I9">
         <v>6</v>
       </c>
-      <c r="M9" s="7"/>
-      <c r="N9" s="7"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
     </row>
     <row r="10" spans="3:16">
       <c r="C10">
@@ -12741,8 +12713,8 @@
       <c r="I10">
         <v>7</v>
       </c>
-      <c r="M10" s="7"/>
-      <c r="N10" s="7"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="3"/>
     </row>
     <row r="11" spans="3:16">
       <c r="C11">
@@ -13058,10 +13030,19 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{829CF65E-34BA-43EF-84E2-8CC1ACB62A83}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61E5803E-A48C-488D-BF94-687FB646AFA7}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>